<commit_message>
Starting design of Controls PCB
</commit_message>
<xml_diff>
--- a/dBu meter calculation.xlsx
+++ b/dBu meter calculation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodri\Documents\GitHub\DMH-Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1745A2BF-F278-4A66-841E-29393780ABAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455815AF-0ACB-4FB8-BF2D-CB7C8CA24C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{34920A5C-097A-4EEA-8361-CAFEEE971C72}"/>
   </bookViews>
@@ -73,7 +73,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,13 +459,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4BAD485-D581-4A2A-9BC3-40AF4B5972F3}">
   <dimension ref="E4:N24"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="10.3984375" customWidth="1"/>
-    <col min="10" max="10" width="15.69921875" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:14">
+    <row r="4" spans="7:14" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
         <v>3</v>
       </c>
@@ -473,7 +473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="7:14">
+    <row r="5" spans="7:14" x14ac:dyDescent="0.3">
       <c r="I5">
         <v>11.7</v>
       </c>
@@ -481,7 +481,7 @@
         <v>56000</v>
       </c>
     </row>
-    <row r="6" spans="7:14">
+    <row r="6" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>0</v>
       </c>
@@ -502,7 +502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="7:14">
+    <row r="7" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G7">
         <v>6</v>
       </c>
@@ -534,7 +534,7 @@
         <v>2.2009500777336326</v>
       </c>
     </row>
-    <row r="8" spans="7:14">
+    <row r="8" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G8">
         <v>3</v>
       </c>
@@ -566,7 +566,7 @@
         <v>1.5339955087234409</v>
       </c>
     </row>
-    <row r="9" spans="7:14">
+    <row r="9" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G9">
         <v>0</v>
       </c>
@@ -598,7 +598,7 @@
         <v>1.0893591293833131</v>
       </c>
     </row>
-    <row r="10" spans="7:14">
+    <row r="10" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G10">
         <v>-3</v>
       </c>
@@ -630,7 +630,7 @@
         <v>0.77407151494213167</v>
       </c>
     </row>
-    <row r="11" spans="7:14">
+    <row r="11" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G11">
         <v>-6</v>
       </c>
@@ -662,7 +662,7 @@
         <v>0.55175332527206766</v>
       </c>
     </row>
-    <row r="12" spans="7:14">
+    <row r="12" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G12">
         <v>-9</v>
       </c>
@@ -694,7 +694,7 @@
         <v>0.38602522024529279</v>
       </c>
     </row>
-    <row r="13" spans="7:14">
+    <row r="13" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G13">
         <v>-12</v>
       </c>
@@ -726,7 +726,7 @@
         <v>0.27284505095871481</v>
       </c>
     </row>
-    <row r="14" spans="7:14">
+    <row r="14" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G14">
         <v>-15</v>
       </c>
@@ -758,7 +758,7 @@
         <v>0.19402314734841938</v>
       </c>
     </row>
-    <row r="15" spans="7:14">
+    <row r="15" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G15">
         <v>-18</v>
       </c>
@@ -790,7 +790,7 @@
         <v>0.13945413715667646</v>
       </c>
     </row>
-    <row r="16" spans="7:14">
+    <row r="16" spans="7:14" x14ac:dyDescent="0.3">
       <c r="G16">
         <v>-21</v>
       </c>
@@ -822,7 +822,7 @@
         <v>9.4990499222663671E-2</v>
       </c>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="3"/>
     </row>
   </sheetData>
@@ -833,13 +833,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E62D02EB-515C-4A0B-BB92-62D83B04599D}">
   <dimension ref="E4:P24"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="10.3984375" customWidth="1"/>
-    <col min="10" max="10" width="15.69921875" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:16">
+    <row r="4" spans="7:16" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
         <v>3</v>
       </c>
@@ -847,7 +847,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="7:16">
+    <row r="5" spans="7:16" x14ac:dyDescent="0.3">
       <c r="I5">
         <v>11.7</v>
       </c>
@@ -855,7 +855,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="6" spans="7:16">
+    <row r="6" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>0</v>
       </c>
@@ -882,7 +882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="7:16">
+    <row r="7" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G7">
         <v>6</v>
       </c>
@@ -922,7 +922,7 @@
         <v>5.8681487239623698</v>
       </c>
     </row>
-    <row r="8" spans="7:16">
+    <row r="8" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G8">
         <v>3</v>
       </c>
@@ -962,7 +962,7 @@
         <v>2.7344688478469674</v>
       </c>
     </row>
-    <row r="9" spans="7:16">
+    <row r="9" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G9">
         <v>0</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>-0.39539566455651648</v>
       </c>
     </row>
-    <row r="10" spans="7:16">
+    <row r="10" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G10">
         <v>-3</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>-3.4975765903157132</v>
       </c>
     </row>
-    <row r="11" spans="7:16">
+    <row r="11" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G11">
         <v>-6</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>-6.8214436555266067</v>
       </c>
     </row>
-    <row r="12" spans="7:16">
+    <row r="12" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G12">
         <v>-9</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>-9.9571657327324985</v>
       </c>
     </row>
-    <row r="13" spans="7:16">
+    <row r="13" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G13">
         <v>-12</v>
       </c>
@@ -1162,7 +1162,7 @@
         <v>-13.49352797102696</v>
       </c>
     </row>
-    <row r="14" spans="7:16">
+    <row r="14" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G14">
         <v>-15</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>-17.125163586105806</v>
       </c>
     </row>
-    <row r="15" spans="7:16">
+    <row r="15" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G15">
         <v>-18</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>-21.408789759382216</v>
       </c>
     </row>
-    <row r="16" spans="7:16">
+    <row r="16" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G16">
         <v>-21</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>-26.028632340506746</v>
       </c>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="3"/>
     </row>
   </sheetData>
@@ -1293,13 +1293,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B938745-C031-44EB-8DE0-C90EAC00962D}">
   <dimension ref="G4:L22"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="10.3984375" customWidth="1"/>
-    <col min="10" max="10" width="15.69921875" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:12">
+    <row r="4" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
         <v>3</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="7:12">
+    <row r="5" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I5">
         <v>10</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="6" spans="7:12">
+    <row r="6" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>0</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="7:12">
+    <row r="7" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G7">
         <v>6</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>2.1937000000000002</v>
       </c>
     </row>
-    <row r="8" spans="7:12">
+    <row r="8" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G8">
         <v>3</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>1.5447</v>
       </c>
     </row>
-    <row r="9" spans="7:12">
+    <row r="9" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G9">
         <v>0</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>1.0917000000000001</v>
       </c>
     </row>
-    <row r="10" spans="7:12">
+    <row r="10" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G10">
         <v>-3</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>0.77570000000000006</v>
       </c>
     </row>
-    <row r="11" spans="7:12">
+    <row r="11" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G11">
         <v>-6</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>0.54969999999999997</v>
       </c>
     </row>
-    <row r="12" spans="7:12">
+    <row r="12" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G12">
         <v>-9</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>0.38769999999999999</v>
       </c>
     </row>
-    <row r="13" spans="7:12">
+    <row r="13" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G13">
         <v>-12</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>0.2747</v>
       </c>
     </row>
-    <row r="14" spans="7:12">
+    <row r="14" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G14">
         <v>-18</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>0.19600000000000001</v>
       </c>
     </row>
-    <row r="15" spans="7:12">
+    <row r="15" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G15">
         <v>-21</v>
       </c>
@@ -1550,22 +1550,22 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="7:12">
+    <row r="16" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I16" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="10:10">
+    <row r="20" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J20">
         <v>76800</v>
       </c>
     </row>
-    <row r="21" spans="10:10">
+    <row r="21" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J21">
         <v>1270</v>
       </c>
     </row>
-    <row r="22" spans="10:10">
+    <row r="22" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J22">
         <f>J21+J20</f>
         <v>78070</v>
@@ -1579,13 +1579,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DFC1236-186E-4F8D-ACF7-7671CAF785F5}">
   <dimension ref="G4:L10"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="10.3984375" customWidth="1"/>
-    <col min="10" max="10" width="15.69921875" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:12">
+    <row r="4" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
         <v>3</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="7:12">
+    <row r="5" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I5">
         <v>11.75</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>104500</v>
       </c>
     </row>
-    <row r="6" spans="7:12">
+    <row r="6" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>0</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="7:12">
+    <row r="7" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G7">
         <v>14</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>5.4533492822966503</v>
       </c>
     </row>
-    <row r="8" spans="7:12">
+    <row r="8" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G8">
         <v>12</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>4.5313397129186601</v>
       </c>
     </row>
-    <row r="9" spans="7:12">
+    <row r="9" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G9">
         <v>-17</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>0.14617224880382776</v>
       </c>
     </row>
-    <row r="10" spans="7:12">
+    <row r="10" spans="7:12" x14ac:dyDescent="0.3">
       <c r="I10" t="s">
         <v>4</v>
       </c>
@@ -1703,14 +1703,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FFD0610-6C73-49A0-8AD5-4029EC3BB905}">
   <dimension ref="E4:P24"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="10.3984375" customWidth="1"/>
-    <col min="10" max="10" width="15.69921875" customWidth="1"/>
-    <col min="16" max="16" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:16">
+    <row r="4" spans="7:16" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
         <v>3</v>
       </c>
@@ -1718,15 +1718,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="7:16">
+    <row r="5" spans="7:16" x14ac:dyDescent="0.3">
       <c r="I5">
-        <v>11.7</v>
+        <v>11.67</v>
       </c>
       <c r="J5">
         <v>100000</v>
       </c>
     </row>
-    <row r="6" spans="7:16">
+    <row r="6" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>0</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="7:16">
+    <row r="7" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G7">
         <v>6</v>
       </c>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="I7" s="1">
         <f t="shared" ref="I7:I14" si="0">H7/$I$5</f>
-        <v>0.18679487179487184</v>
+        <v>0.18727506426735221</v>
       </c>
       <c r="J7" s="4">
         <v>5600</v>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="L7" s="1">
         <f t="shared" ref="L7:L16" si="1">K7*$I$5</f>
-        <v>2.2171499999999997</v>
+        <v>2.211465</v>
       </c>
       <c r="M7" s="1">
         <f>SUM(J7:J16)/SUM(J6:J16)</f>
@@ -1782,18 +1782,18 @@
       </c>
       <c r="N7" s="1">
         <f>M7*$I$5</f>
-        <v>2.1962852897473994</v>
+        <v>2.1906537890044575</v>
       </c>
       <c r="O7" s="1">
         <f>N7/SQRT(2)</f>
-        <v>1.5530082218006473</v>
+        <v>1.5490261494370561</v>
       </c>
       <c r="P7" s="1">
         <f>20*LOG10(O7/0.7746)</f>
-        <v>6.0419252457708001</v>
-      </c>
-    </row>
-    <row r="8" spans="7:16">
+        <v>6.0196251317549727</v>
+      </c>
+    </row>
+    <row r="8" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G8">
         <v>3</v>
       </c>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
-        <v>0.13226495726495729</v>
+        <v>0.132604970008569</v>
       </c>
       <c r="J8" s="4">
         <v>3900</v>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="L8" s="1">
         <f t="shared" si="1"/>
-        <v>1.5619499999999999</v>
+        <v>1.5579450000000001</v>
       </c>
       <c r="M8" s="1">
         <f>SUM(J8:J16)/SUM(J6:J16)</f>
@@ -1822,18 +1822,18 @@
       </c>
       <c r="N8" s="1">
         <f t="shared" ref="N8:N16" si="2">M8*$I$5</f>
-        <v>1.5472511144130756</v>
+        <v>1.5432838038632988</v>
       </c>
       <c r="O8" s="1">
         <f t="shared" ref="O8:O16" si="3">N8/SQRT(2)</f>
-        <v>1.0940717551999284</v>
+        <v>1.0912664430071082</v>
       </c>
       <c r="P8" s="1">
         <f t="shared" ref="P8:P16" si="4">20*LOG10(O8/0.7746)</f>
-        <v>2.9993662737008591</v>
-      </c>
-    </row>
-    <row r="9" spans="7:16">
+        <v>2.9770661596850307</v>
+      </c>
+    </row>
+    <row r="9" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G9">
         <v>0</v>
       </c>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
-        <v>9.358974358974359E-2</v>
+        <v>9.383033419023136E-2</v>
       </c>
       <c r="J9" s="4">
         <v>2700</v>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="L9" s="1">
         <f t="shared" si="1"/>
-        <v>1.10565</v>
+        <v>1.1028150000000001</v>
       </c>
       <c r="M9" s="1">
         <f>SUM(J9:J16)/SUM(J6:J16)</f>
@@ -1862,18 +1862,18 @@
       </c>
       <c r="N9" s="1">
         <f t="shared" si="2"/>
-        <v>1.0952451708766715</v>
+        <v>1.0924368499257058</v>
       </c>
       <c r="O9" s="1">
         <f t="shared" si="3"/>
-        <v>0.77445528738871339</v>
+        <v>0.7724695046005372</v>
       </c>
       <c r="P9" s="1">
         <f t="shared" si="4"/>
-        <v>-1.6228701257612276E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="7:16">
+        <v>-2.3922984141590359E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G10">
         <v>-3</v>
       </c>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="I10" s="1">
         <f t="shared" si="0"/>
-        <v>6.628205128205128E-2</v>
+        <v>6.6452442159383035E-2</v>
       </c>
       <c r="J10" s="4">
         <v>2000</v>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="L10" s="1">
         <f t="shared" si="1"/>
-        <v>0.78974999999999995</v>
+        <v>0.78772500000000001</v>
       </c>
       <c r="M10" s="1">
         <f>SUM(J10:J16)/SUM(J6:J16)</f>
@@ -1902,18 +1902,18 @@
       </c>
       <c r="N10" s="1">
         <f t="shared" si="2"/>
-        <v>0.78231797919762247</v>
+        <v>0.78031203566121843</v>
       </c>
       <c r="O10" s="1">
         <f t="shared" si="3"/>
-        <v>0.55318234813479528</v>
+        <v>0.55176393185752659</v>
       </c>
       <c r="P10" s="1">
         <f t="shared" si="4"/>
-        <v>-2.9241835836905223</v>
-      </c>
-    </row>
-    <row r="11" spans="7:16">
+        <v>-2.9464836977063507</v>
+      </c>
+    </row>
+    <row r="11" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G11">
         <v>-6</v>
       </c>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="I11" s="1">
         <f t="shared" si="0"/>
-        <v>4.6923076923076928E-2</v>
+        <v>4.7043701799485867E-2</v>
       </c>
       <c r="J11" s="4">
         <v>1390</v>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="L11" s="1">
         <f t="shared" si="1"/>
-        <v>0.55574999999999997</v>
+        <v>0.55432499999999996</v>
       </c>
       <c r="M11" s="1">
         <f>SUM(J11:J16)/SUM(J6:J16)</f>
@@ -1942,18 +1942,18 @@
       </c>
       <c r="N11" s="1">
         <f t="shared" si="2"/>
-        <v>0.55052005943536397</v>
+        <v>0.54910846953937587</v>
       </c>
       <c r="O11" s="1">
         <f t="shared" si="3"/>
-        <v>0.38927646720596704</v>
+        <v>0.38827832241825944</v>
       </c>
       <c r="P11" s="1">
         <f t="shared" si="4"/>
-        <v>-5.9763868478136883</v>
-      </c>
-    </row>
-    <row r="12" spans="7:16">
+        <v>-5.9986869618295193</v>
+      </c>
+    </row>
+    <row r="12" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G12">
         <v>-9</v>
       </c>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="I12" s="1">
         <f t="shared" si="0"/>
-        <v>3.3205128205128207E-2</v>
+        <v>3.3290488431876611E-2</v>
       </c>
       <c r="J12" s="4">
         <v>1000</v>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="L12" s="1">
         <f t="shared" si="1"/>
-        <v>0.39311999999999997</v>
+        <v>0.39211199999999996</v>
       </c>
       <c r="M12" s="1">
         <f>SUM(J12:J16)/SUM(J6:J16)</f>
@@ -1982,18 +1982,18 @@
       </c>
       <c r="N12" s="1">
         <f t="shared" si="2"/>
-        <v>0.38942050520059435</v>
+        <v>0.38842199108469538</v>
       </c>
       <c r="O12" s="1">
         <f t="shared" si="3"/>
-        <v>0.27536187996043143</v>
+        <v>0.27465582385796877</v>
       </c>
       <c r="P12" s="1">
         <f t="shared" si="4"/>
-        <v>-8.9834734925141397</v>
-      </c>
-    </row>
-    <row r="13" spans="7:16">
+        <v>-9.0057736065299689</v>
+      </c>
+    </row>
+    <row r="13" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G13">
         <v>-12</v>
       </c>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="I13" s="1">
         <f t="shared" si="0"/>
-        <v>2.3504273504273508E-2</v>
+        <v>2.3564695801199659E-2</v>
       </c>
       <c r="J13" s="4">
         <v>1200</v>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="L13" s="1">
         <f t="shared" si="1"/>
-        <v>0.27611999999999998</v>
+        <v>0.27541199999999999</v>
       </c>
       <c r="M13" s="1">
         <f>SUM(J13:J16)/SUM(J6:J16)</f>
@@ -2022,18 +2022,18 @@
       </c>
       <c r="N13" s="1">
         <f t="shared" si="2"/>
-        <v>0.27352154531946504</v>
+        <v>0.27282020802377416</v>
       </c>
       <c r="O13" s="1">
         <f t="shared" si="3"/>
-        <v>0.19340893949601728</v>
+        <v>0.19291301913833525</v>
       </c>
       <c r="P13" s="1">
         <f t="shared" si="4"/>
-        <v>-12.05201898090889</v>
-      </c>
-    </row>
-    <row r="14" spans="7:16">
+        <v>-12.074319094924718</v>
+      </c>
+    </row>
+    <row r="14" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G14">
         <v>-15</v>
       </c>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="I14" s="1">
         <f t="shared" si="0"/>
-        <v>1.666666666666667E-2</v>
+        <v>1.6709511568123395E-2</v>
       </c>
       <c r="J14" s="4">
         <v>560</v>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="L14" s="1">
         <f t="shared" si="1"/>
-        <v>0.13571999999999998</v>
+        <v>0.13537199999999999</v>
       </c>
       <c r="M14" s="1">
         <f>SUM(J14:J16)/SUM(J6:J16)</f>
@@ -2062,18 +2062,18 @@
       </c>
       <c r="N14" s="1">
         <f t="shared" si="2"/>
-        <v>0.13444279346210997</v>
+        <v>0.13409806835066865</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" si="3"/>
-        <v>9.5065410938720382E-2</v>
+        <v>9.4821653474774947E-2</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" si="4"/>
-        <v>-18.22109925577265</v>
-      </c>
-    </row>
-    <row r="15" spans="7:16">
+        <v>-18.243399369788481</v>
+      </c>
+    </row>
+    <row r="15" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G15">
         <v>-18</v>
       </c>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="I15" s="1">
         <f>H15/$I$5</f>
-        <v>1.1794871794871797E-2</v>
+        <v>1.1825192802056557E-2</v>
       </c>
       <c r="J15" s="4">
         <v>330</v>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="L15" s="1">
         <f t="shared" si="1"/>
-        <v>8.5609756097560982E-2</v>
+        <v>8.5390243902439031E-2</v>
       </c>
       <c r="M15" s="1">
         <f>SUM(J15:J16)/SUM(J6:J16)</f>
@@ -2102,18 +2102,18 @@
       </c>
       <c r="N15" s="1">
         <f t="shared" si="2"/>
-        <v>6.9539375928677552E-2</v>
+        <v>6.9361069836552741E-2</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" si="3"/>
-        <v>4.9171764278648465E-2</v>
+        <v>4.9045682831780138E-2</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" si="4"/>
-        <v>-23.947234032638146</v>
-      </c>
-    </row>
-    <row r="16" spans="7:16">
+        <v>-23.969534146653974</v>
+      </c>
+    </row>
+    <row r="16" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G16">
         <v>-21</v>
       </c>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="I16" s="1">
         <f>H16/$I$5</f>
-        <v>8.333333333333335E-3</v>
+        <v>8.3547557840616977E-3</v>
       </c>
       <c r="J16" s="4">
         <v>270</v>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="L16" s="1">
         <f t="shared" si="1"/>
-        <v>3.159E-2</v>
+        <v>3.1509000000000002E-2</v>
       </c>
       <c r="M16" s="1">
         <f>SUM(J16)/SUM(J6:J16)</f>
@@ -2142,18 +2142,18 @@
       </c>
       <c r="N16" s="1">
         <f t="shared" si="2"/>
-        <v>3.1292719167904902E-2</v>
+        <v>3.1212481426448738E-2</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" si="3"/>
-        <v>2.2127293925391811E-2</v>
+        <v>2.2070557274301066E-2</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" si="4"/>
-        <v>-30.882983757131271</v>
-      </c>
-    </row>
-    <row r="24" spans="5:5">
+        <v>-30.905283871147105</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simulated 10V ref for VU meter
</commit_message>
<xml_diff>
--- a/dBu meter calculation.xlsx
+++ b/dBu meter calculation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodri\Documents\GitHub\DMH-Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455815AF-0ACB-4FB8-BF2D-CB7C8CA24C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D563AD1F-5818-47CF-B116-FF3C5ECCD93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{34920A5C-097A-4EEA-8361-CAFEEE971C72}"/>
   </bookViews>
@@ -18,6 +18,8 @@
     <sheet name="10V" sheetId="3" r:id="rId3"/>
     <sheet name="In 11v75" sheetId="5" r:id="rId4"/>
     <sheet name="Out 11v70 (2)" sheetId="7" r:id="rId5"/>
+    <sheet name="Out 10V" sheetId="8" r:id="rId6"/>
+    <sheet name="Out 10V (2)" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="8">
   <si>
     <t>dBu</t>
   </si>
@@ -1770,27 +1772,27 @@
       </c>
       <c r="K7" s="1">
         <f>SUM(J7:J16)/J5</f>
-        <v>0.1895</v>
+        <v>0.18970000000000001</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" ref="L7:L16" si="1">K7*$I$5</f>
-        <v>2.211465</v>
+        <v>2.2137990000000003</v>
       </c>
       <c r="M7" s="1">
         <f>SUM(J7:J16)/SUM(J6:J16)</f>
-        <v>0.18771669143140168</v>
+        <v>0.18787758740219868</v>
       </c>
       <c r="N7" s="1">
         <f>M7*$I$5</f>
-        <v>2.1906537890044575</v>
+        <v>2.1925314449836586</v>
       </c>
       <c r="O7" s="1">
         <f>N7/SQRT(2)</f>
-        <v>1.5490261494370561</v>
+        <v>1.5503538527126846</v>
       </c>
       <c r="P7" s="1">
         <f>20*LOG10(O7/0.7746)</f>
-        <v>6.0196251317549727</v>
+        <v>6.0270668038452779</v>
       </c>
     </row>
     <row r="8" spans="7:16" x14ac:dyDescent="0.3">
@@ -1810,27 +1812,27 @@
       </c>
       <c r="K8" s="1">
         <f>SUM(J8:J16)/J5</f>
-        <v>0.13350000000000001</v>
+        <v>0.13370000000000001</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" si="1"/>
-        <v>1.5579450000000001</v>
+        <v>1.5602790000000002</v>
       </c>
       <c r="M8" s="1">
         <f>SUM(J8:J16)/SUM(J6:J16)</f>
-        <v>0.13224368499257058</v>
+        <v>0.13241556898088541</v>
       </c>
       <c r="N8" s="1">
         <f t="shared" ref="N8:N16" si="2">M8*$I$5</f>
-        <v>1.5432838038632988</v>
+        <v>1.5452896900069328</v>
       </c>
       <c r="O8" s="1">
         <f t="shared" ref="O8:O16" si="3">N8/SQRT(2)</f>
-        <v>1.0912664430071082</v>
+        <v>1.0926848187015601</v>
       </c>
       <c r="P8" s="1">
         <f t="shared" ref="P8:P16" si="4">20*LOG10(O8/0.7746)</f>
-        <v>2.9770661596850307</v>
+        <v>2.9883483313117152</v>
       </c>
     </row>
     <row r="9" spans="7:16" x14ac:dyDescent="0.3">
@@ -1850,27 +1852,27 @@
       </c>
       <c r="K9" s="1">
         <f>SUM(J9:J16)/J5</f>
-        <v>9.4500000000000001E-2</v>
+        <v>9.4700000000000006E-2</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="1"/>
-        <v>1.1028150000000001</v>
+        <v>1.1051490000000002</v>
       </c>
       <c r="M9" s="1">
         <f>SUM(J9:J16)/SUM(J6:J16)</f>
-        <v>9.3610698365527489E-2</v>
+        <v>9.3790234723185109E-2</v>
       </c>
       <c r="N9" s="1">
         <f t="shared" si="2"/>
-        <v>1.0924368499257058</v>
+        <v>1.0945320392195703</v>
       </c>
       <c r="O9" s="1">
         <f t="shared" si="3"/>
-        <v>0.7724695046005372</v>
+        <v>0.77395102715809827</v>
       </c>
       <c r="P9" s="1">
         <f t="shared" si="4"/>
-        <v>-2.3922984141590359E-2</v>
+        <v>-7.2802338625028301E-3</v>
       </c>
     </row>
     <row r="10" spans="7:16" x14ac:dyDescent="0.3">
@@ -1890,27 +1892,27 @@
       </c>
       <c r="K10" s="1">
         <f>SUM(J10:J16)/J5</f>
-        <v>6.7500000000000004E-2</v>
+        <v>6.7699999999999996E-2</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="1"/>
-        <v>0.78772500000000001</v>
+        <v>0.79005899999999996</v>
       </c>
       <c r="M10" s="1">
         <f>SUM(J10:J16)/SUM(J6:J16)</f>
-        <v>6.6864784546805348E-2</v>
+        <v>6.7049618698623359E-2</v>
       </c>
       <c r="N10" s="1">
         <f t="shared" si="2"/>
-        <v>0.78031203566121843</v>
+        <v>0.78246905021293456</v>
       </c>
       <c r="O10" s="1">
         <f t="shared" si="3"/>
-        <v>0.55176393185752659</v>
+        <v>0.55328917147416312</v>
       </c>
       <c r="P10" s="1">
         <f t="shared" si="4"/>
-        <v>-2.9464836977063507</v>
+        <v>-2.9225064402250855</v>
       </c>
     </row>
     <row r="11" spans="7:16" x14ac:dyDescent="0.3">
@@ -1930,27 +1932,27 @@
       </c>
       <c r="K11" s="1">
         <f>SUM(J11:J16)/J5</f>
-        <v>4.7500000000000001E-2</v>
+        <v>4.7699999999999999E-2</v>
       </c>
       <c r="L11" s="1">
         <f t="shared" si="1"/>
-        <v>0.55432499999999996</v>
+        <v>0.55665900000000001</v>
       </c>
       <c r="M11" s="1">
         <f>SUM(J11:J16)/SUM(J6:J16)</f>
-        <v>4.7052996532937097E-2</v>
+        <v>4.724175497672576E-2</v>
       </c>
       <c r="N11" s="1">
         <f t="shared" si="2"/>
-        <v>0.54910846953937587</v>
+        <v>0.55131128057838963</v>
       </c>
       <c r="O11" s="1">
         <f t="shared" si="3"/>
-        <v>0.38827832241825944</v>
+        <v>0.38983594504161861</v>
       </c>
       <c r="P11" s="1">
         <f t="shared" si="4"/>
-        <v>-5.9986869618295193</v>
+        <v>-5.9639122331256935</v>
       </c>
     </row>
     <row r="12" spans="7:16" x14ac:dyDescent="0.3">
@@ -1970,27 +1972,27 @@
       </c>
       <c r="K12" s="1">
         <f>SUM(J12:J16)/J5</f>
-        <v>3.3599999999999998E-2</v>
+        <v>3.3799999999999997E-2</v>
       </c>
       <c r="L12" s="1">
         <f t="shared" si="1"/>
-        <v>0.39211199999999996</v>
+        <v>0.39444599999999996</v>
       </c>
       <c r="M12" s="1">
         <f>SUM(J12:J16)/SUM(J6:J16)</f>
-        <v>3.3283803863298662E-2</v>
+        <v>3.3475289690006932E-2</v>
       </c>
       <c r="N12" s="1">
         <f t="shared" si="2"/>
-        <v>0.38842199108469538</v>
+        <v>0.39065663068238088</v>
       </c>
       <c r="O12" s="1">
         <f t="shared" si="3"/>
-        <v>0.27465582385796877</v>
+        <v>0.27623595267100021</v>
       </c>
       <c r="P12" s="1">
         <f t="shared" si="4"/>
-        <v>-9.0057736065299689</v>
+        <v>-8.955945808374878</v>
       </c>
     </row>
     <row r="13" spans="7:16" x14ac:dyDescent="0.3">
@@ -2006,31 +2008,31 @@
         <v>2.3564695801199659E-2</v>
       </c>
       <c r="J13" s="4">
-        <v>1200</v>
+        <v>1220</v>
       </c>
       <c r="K13" s="1">
         <f>SUM(J13:J16)/J5</f>
-        <v>2.3599999999999999E-2</v>
+        <v>2.3800000000000002E-2</v>
       </c>
       <c r="L13" s="1">
         <f t="shared" si="1"/>
-        <v>0.27541199999999999</v>
+        <v>0.27774599999999999</v>
       </c>
       <c r="M13" s="1">
         <f>SUM(J13:J16)/SUM(J6:J16)</f>
-        <v>2.3377909856364537E-2</v>
+        <v>2.3571357829058136E-2</v>
       </c>
       <c r="N13" s="1">
         <f t="shared" si="2"/>
-        <v>0.27282020802377416</v>
+        <v>0.27507774586510847</v>
       </c>
       <c r="O13" s="1">
         <f t="shared" si="3"/>
-        <v>0.19291301913833525</v>
+        <v>0.19450933945472798</v>
       </c>
       <c r="P13" s="1">
         <f t="shared" si="4"/>
-        <v>-12.074319094924718</v>
+        <v>-12.002740672797731</v>
       </c>
     </row>
     <row r="14" spans="7:16" x14ac:dyDescent="0.3">
@@ -2058,19 +2060,19 @@
       </c>
       <c r="M14" s="1">
         <f>SUM(J14:J16)/SUM(J6:J16)</f>
-        <v>1.1490837048043587E-2</v>
+        <v>1.1488560958700603E-2</v>
       </c>
       <c r="N14" s="1">
         <f t="shared" si="2"/>
-        <v>0.13409806835066865</v>
+        <v>0.13407150638803603</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" si="3"/>
-        <v>9.4821653474774947E-2</v>
+        <v>9.4802871330875796E-2</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" si="4"/>
-        <v>-18.243399369788481</v>
+        <v>-18.245120029389604</v>
       </c>
     </row>
     <row r="15" spans="7:16" x14ac:dyDescent="0.3">
@@ -2098,19 +2100,19 @@
       </c>
       <c r="M15" s="1">
         <f>SUM(J15:J16)/SUM(J6:J16)</f>
-        <v>5.9435364041604752E-3</v>
+        <v>5.942359116569278E-3</v>
       </c>
       <c r="N15" s="1">
         <f t="shared" si="2"/>
-        <v>6.9361069836552741E-2</v>
+        <v>6.9347330890363476E-2</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" si="3"/>
-        <v>4.9045682831780138E-2</v>
+        <v>4.9035967929763349E-2</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" si="4"/>
-        <v>-23.969534146653974</v>
+        <v>-23.9712548062551</v>
       </c>
     </row>
     <row r="16" spans="7:16" x14ac:dyDescent="0.3">
@@ -2138,19 +2140,941 @@
       </c>
       <c r="M16" s="1">
         <f>SUM(J16)/SUM(J6:J16)</f>
-        <v>2.674591381872214E-3</v>
+        <v>2.6740616024561749E-3</v>
       </c>
       <c r="N16" s="1">
         <f t="shared" si="2"/>
-        <v>3.1212481426448738E-2</v>
+        <v>3.1206298900663561E-2</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" si="3"/>
-        <v>2.2070557274301066E-2</v>
+        <v>2.2066185568393504E-2</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" si="4"/>
-        <v>-30.905283871147105</v>
+        <v>-30.907004530748225</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E24" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{828C9D39-9CEC-4B02-9287-72FBA31A5E5E}">
+  <dimension ref="E4:P24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="6" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="3">
+        <v>82000</v>
+      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N6" t="s">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
+        <v>6</v>
+      </c>
+      <c r="P6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7" s="1">
+        <f>4.371/2</f>
+        <v>2.1855000000000002</v>
+      </c>
+      <c r="I7" s="1">
+        <f t="shared" ref="I7:I14" si="0">H7/$I$5</f>
+        <v>0.21855000000000002</v>
+      </c>
+      <c r="J7" s="4">
+        <v>6800</v>
+      </c>
+      <c r="K7" s="1">
+        <f>SUM(J7:J16)/J5</f>
+        <v>0.2296</v>
+      </c>
+      <c r="L7" s="1">
+        <f t="shared" ref="L7:L16" si="1">K7*$I$5</f>
+        <v>2.2959999999999998</v>
+      </c>
+      <c r="M7" s="1">
+        <f>SUM(J7:J16)/SUM(J6:J16)</f>
+        <v>0.21875</v>
+      </c>
+      <c r="N7" s="1">
+        <f>M7*$I$5</f>
+        <v>2.1875</v>
+      </c>
+      <c r="O7" s="1">
+        <f>N7/SQRT(2)</f>
+        <v>1.5467960838455725</v>
+      </c>
+      <c r="P7" s="1">
+        <f>20*LOG10(O7/0.7746)</f>
+        <v>6.0071114242459256</v>
+      </c>
+    </row>
+    <row r="8" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" s="1">
+        <f>3.095/2</f>
+        <v>1.5475000000000001</v>
+      </c>
+      <c r="I8" s="1">
+        <f t="shared" si="0"/>
+        <v>0.15475</v>
+      </c>
+      <c r="J8" s="4">
+        <v>4700</v>
+      </c>
+      <c r="K8" s="1">
+        <f>SUM(J8:J16)/J5</f>
+        <v>0.16159999999999999</v>
+      </c>
+      <c r="L8" s="1">
+        <f t="shared" si="1"/>
+        <v>1.6159999999999999</v>
+      </c>
+      <c r="M8" s="1">
+        <f>SUM(J8:J16)/SUM(J6:J16)</f>
+        <v>0.15396341463414634</v>
+      </c>
+      <c r="N8" s="1">
+        <f t="shared" ref="N8:N16" si="2">M8*$I$5</f>
+        <v>1.5396341463414633</v>
+      </c>
+      <c r="O8" s="1">
+        <f t="shared" ref="O8:O16" si="3">N8/SQRT(2)</f>
+        <v>1.0886857454244099</v>
+      </c>
+      <c r="P8" s="1">
+        <f t="shared" ref="P8:P16" si="4">20*LOG10(O8/0.7746)</f>
+        <v>2.9565008784985549</v>
+      </c>
+    </row>
+    <row r="9" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <f>2.19/2</f>
+        <v>1.095</v>
+      </c>
+      <c r="I9" s="1">
+        <f t="shared" si="0"/>
+        <v>0.1095</v>
+      </c>
+      <c r="J9" s="4">
+        <v>3300</v>
+      </c>
+      <c r="K9" s="1">
+        <f>SUM(J9:J16)/J5</f>
+        <v>0.11459999999999999</v>
+      </c>
+      <c r="L9" s="1">
+        <f t="shared" si="1"/>
+        <v>1.1459999999999999</v>
+      </c>
+      <c r="M9" s="1">
+        <f>SUM(J9:J16)/SUM(J6:J16)</f>
+        <v>0.1091844512195122</v>
+      </c>
+      <c r="N9" s="1">
+        <f t="shared" si="2"/>
+        <v>1.0918445121951219</v>
+      </c>
+      <c r="O9" s="1">
+        <f t="shared" si="3"/>
+        <v>0.77205065857448874</v>
+      </c>
+      <c r="P9" s="1">
+        <f t="shared" si="4"/>
+        <v>-2.8633897645368452E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <v>-3</v>
+      </c>
+      <c r="H10" s="1">
+        <f>1.551/2</f>
+        <v>0.77549999999999997</v>
+      </c>
+      <c r="I10" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7549999999999994E-2</v>
+      </c>
+      <c r="J10" s="4">
+        <v>2390</v>
+      </c>
+      <c r="K10" s="1">
+        <f>SUM(J10:J16)/J5</f>
+        <v>8.1600000000000006E-2</v>
+      </c>
+      <c r="L10" s="1">
+        <f t="shared" si="1"/>
+        <v>0.81600000000000006</v>
+      </c>
+      <c r="M10" s="1">
+        <f>SUM(J10:J16)/SUM(J6:J16)</f>
+        <v>7.774390243902439E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <f t="shared" si="2"/>
+        <v>0.77743902439024393</v>
+      </c>
+      <c r="O10" s="1">
+        <f t="shared" si="3"/>
+        <v>0.5497324061053952</v>
+      </c>
+      <c r="P10" s="1">
+        <f t="shared" si="4"/>
+        <v>-2.9785230751955689</v>
+      </c>
+    </row>
+    <row r="11" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <v>-6</v>
+      </c>
+      <c r="H11">
+        <f>1.098/2</f>
+        <v>0.54900000000000004</v>
+      </c>
+      <c r="I11" s="1">
+        <f t="shared" si="0"/>
+        <v>5.4900000000000004E-2</v>
+      </c>
+      <c r="J11" s="4">
+        <v>1680</v>
+      </c>
+      <c r="K11" s="1">
+        <f>SUM(J11:J16)/J5</f>
+        <v>5.7700000000000001E-2</v>
+      </c>
+      <c r="L11" s="1">
+        <f t="shared" si="1"/>
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="M11" s="1">
+        <f>SUM(J11:J16)/SUM(J6:J16)</f>
+        <v>5.4973323170731704E-2</v>
+      </c>
+      <c r="N11" s="1">
+        <f t="shared" si="2"/>
+        <v>0.54973323170731703</v>
+      </c>
+      <c r="O11" s="1">
+        <f t="shared" si="3"/>
+        <v>0.38872009598383944</v>
+      </c>
+      <c r="P11" s="1">
+        <f t="shared" si="4"/>
+        <v>-5.988809987158163</v>
+      </c>
+    </row>
+    <row r="12" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>-9</v>
+      </c>
+      <c r="H12" s="1">
+        <f>0.777/2</f>
+        <v>0.38850000000000001</v>
+      </c>
+      <c r="I12" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8850000000000003E-2</v>
+      </c>
+      <c r="J12" s="4">
+        <v>1220</v>
+      </c>
+      <c r="K12" s="1">
+        <f>SUM(J12:J16)/J5</f>
+        <v>4.0899999999999999E-2</v>
+      </c>
+      <c r="L12" s="1">
+        <f t="shared" si="1"/>
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="M12" s="1">
+        <f>SUM(J12:J16)/SUM(J6:J16)</f>
+        <v>3.8967225609756101E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <f t="shared" si="2"/>
+        <v>0.38967225609756101</v>
+      </c>
+      <c r="O12" s="1">
+        <f t="shared" si="3"/>
+        <v>0.27553989472684637</v>
+      </c>
+      <c r="P12" s="1">
+        <f t="shared" si="4"/>
+        <v>-8.9778600901259544</v>
+      </c>
+    </row>
+    <row r="13" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <v>-12</v>
+      </c>
+      <c r="H13">
+        <f>0.55/2</f>
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="I13" s="1">
+        <f t="shared" si="0"/>
+        <v>2.7500000000000004E-2</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1470</v>
+      </c>
+      <c r="K13" s="1">
+        <f>SUM(J13:J16)/J5</f>
+        <v>2.87E-2</v>
+      </c>
+      <c r="L13" s="1">
+        <f t="shared" si="1"/>
+        <v>0.28699999999999998</v>
+      </c>
+      <c r="M13" s="1">
+        <f>SUM(J13:J16)/SUM(J6:J16)</f>
+        <v>2.734375E-2</v>
+      </c>
+      <c r="N13" s="1">
+        <f t="shared" si="2"/>
+        <v>0.2734375</v>
+      </c>
+      <c r="O13" s="1">
+        <f t="shared" si="3"/>
+        <v>0.19334951048069657</v>
+      </c>
+      <c r="P13" s="1">
+        <f t="shared" si="4"/>
+        <v>-12.054688315592944</v>
+      </c>
+    </row>
+    <row r="14" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G14">
+        <v>-15</v>
+      </c>
+      <c r="H14">
+        <f>0.39/2</f>
+        <v>0.19500000000000001</v>
+      </c>
+      <c r="I14" s="1">
+        <f t="shared" si="0"/>
+        <v>1.95E-2</v>
+      </c>
+      <c r="J14" s="4">
+        <v>680</v>
+      </c>
+      <c r="K14" s="1">
+        <f>SUM(J14:J16)/J5</f>
+        <v>1.4E-2</v>
+      </c>
+      <c r="L14" s="1">
+        <f t="shared" si="1"/>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="M14" s="1">
+        <f>SUM(J14:J16)/SUM(J6:J16)</f>
+        <v>1.3338414634146341E-2</v>
+      </c>
+      <c r="N14" s="1">
+        <f t="shared" si="2"/>
+        <v>0.13338414634146342</v>
+      </c>
+      <c r="O14" s="1">
+        <f t="shared" si="3"/>
+        <v>9.4316834380827608E-2</v>
+      </c>
+      <c r="P14" s="1">
+        <f t="shared" si="4"/>
+        <v>-18.289765536708028</v>
+      </c>
+    </row>
+    <row r="15" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G15">
+        <v>-18</v>
+      </c>
+      <c r="H15">
+        <f>0.276/2</f>
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="I15" s="1">
+        <f>H15/$I$5</f>
+        <v>1.3800000000000002E-2</v>
+      </c>
+      <c r="J15" s="4">
+        <v>360</v>
+      </c>
+      <c r="K15" s="1">
+        <f>SUM(J15:J16)/J6</f>
+        <v>8.7804878048780496E-3</v>
+      </c>
+      <c r="L15" s="1">
+        <f t="shared" si="1"/>
+        <v>8.7804878048780496E-2</v>
+      </c>
+      <c r="M15" s="1">
+        <f>SUM(J15:J16)/SUM(J6:J16)</f>
+        <v>6.8597560975609756E-3</v>
+      </c>
+      <c r="N15" s="1">
+        <f t="shared" si="2"/>
+        <v>6.8597560975609762E-2</v>
+      </c>
+      <c r="O15" s="1">
+        <f t="shared" si="3"/>
+        <v>4.8505800538711341E-2</v>
+      </c>
+      <c r="P15" s="1">
+        <f t="shared" si="4"/>
+        <v>-24.065676321647423</v>
+      </c>
+    </row>
+    <row r="16" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G16">
+        <v>-21</v>
+      </c>
+      <c r="H16" s="1">
+        <f>0.195/2</f>
+        <v>9.7500000000000003E-2</v>
+      </c>
+      <c r="I16" s="1">
+        <f>H16/$I$5</f>
+        <v>9.75E-3</v>
+      </c>
+      <c r="J16" s="4">
+        <v>360</v>
+      </c>
+      <c r="K16" s="1">
+        <f t="shared" ref="K16" si="5">J16/$J$5</f>
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="L16" s="1">
+        <f t="shared" si="1"/>
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="M16" s="1">
+        <f>SUM(J16)/SUM(J6:J16)</f>
+        <v>3.4298780487804878E-3</v>
+      </c>
+      <c r="N16" s="1">
+        <f t="shared" si="2"/>
+        <v>3.4298780487804881E-2</v>
+      </c>
+      <c r="O16" s="1">
+        <f t="shared" si="3"/>
+        <v>2.4252900269355671E-2</v>
+      </c>
+      <c r="P16" s="1">
+        <f t="shared" si="4"/>
+        <v>-30.086276234927048</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E24" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C588607-A81A-441B-A5D7-EC57AD3B650D}">
+  <dimension ref="E4:P24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="6" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="3">
+        <v>90900</v>
+      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N6" t="s">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
+        <v>6</v>
+      </c>
+      <c r="P6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7" s="1">
+        <f>4.371/2</f>
+        <v>2.1855000000000002</v>
+      </c>
+      <c r="I7" s="1">
+        <f t="shared" ref="I7:I14" si="0">H7/$I$5</f>
+        <v>0.21855000000000002</v>
+      </c>
+      <c r="J7" s="4">
+        <v>7500</v>
+      </c>
+      <c r="K7" s="1">
+        <f>SUM(J7:J16)/J5</f>
+        <v>0.25979999999999998</v>
+      </c>
+      <c r="L7" s="1">
+        <f t="shared" ref="L7:L16" si="1">K7*$I$5</f>
+        <v>2.5979999999999999</v>
+      </c>
+      <c r="M7" s="1">
+        <f>SUM(J7:J16)/SUM(J6:J16)</f>
+        <v>0.22227926078028748</v>
+      </c>
+      <c r="N7" s="1">
+        <f>M7*$I$5</f>
+        <v>2.2227926078028748</v>
+      </c>
+      <c r="O7" s="1">
+        <f>N7/SQRT(2)</f>
+        <v>1.5717517261487426</v>
+      </c>
+      <c r="P7" s="1">
+        <f>20*LOG10(O7/0.7746)</f>
+        <v>6.1461290665742832</v>
+      </c>
+    </row>
+    <row r="8" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" s="1">
+        <f>3.095/2</f>
+        <v>1.5475000000000001</v>
+      </c>
+      <c r="I8" s="1">
+        <f t="shared" si="0"/>
+        <v>0.15475</v>
+      </c>
+      <c r="J8" s="4">
+        <v>5600</v>
+      </c>
+      <c r="K8" s="1">
+        <f>SUM(J8:J16)/J5</f>
+        <v>0.18479999999999999</v>
+      </c>
+      <c r="L8" s="1">
+        <f t="shared" si="1"/>
+        <v>1.8479999999999999</v>
+      </c>
+      <c r="M8" s="1">
+        <f>SUM(J8:J16)/SUM(J6:J16)</f>
+        <v>0.15811088295687886</v>
+      </c>
+      <c r="N8" s="1">
+        <f t="shared" ref="N8:N16" si="2">M8*$I$5</f>
+        <v>1.5811088295687887</v>
+      </c>
+      <c r="O8" s="1">
+        <f t="shared" ref="O8:O16" si="3">N8/SQRT(2)</f>
+        <v>1.1180127751820157</v>
+      </c>
+      <c r="P8" s="1">
+        <f t="shared" ref="P8:P16" si="4">20*LOG10(O8/0.7746)</f>
+        <v>3.1873854695158617</v>
+      </c>
+    </row>
+    <row r="9" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <f>2.19/2</f>
+        <v>1.095</v>
+      </c>
+      <c r="I9" s="1">
+        <f t="shared" si="0"/>
+        <v>0.1095</v>
+      </c>
+      <c r="J9" s="4">
+        <v>3900</v>
+      </c>
+      <c r="K9" s="1">
+        <f>SUM(J9:J16)/J5</f>
+        <v>0.1288</v>
+      </c>
+      <c r="L9" s="1">
+        <f t="shared" si="1"/>
+        <v>1.288</v>
+      </c>
+      <c r="M9" s="1">
+        <f>SUM(J9:J16)/SUM(J6:J16)</f>
+        <v>0.11019849418206708</v>
+      </c>
+      <c r="N9" s="1">
+        <f t="shared" si="2"/>
+        <v>1.1019849418206709</v>
+      </c>
+      <c r="O9" s="1">
+        <f t="shared" si="3"/>
+        <v>0.77922102512685931</v>
+      </c>
+      <c r="P9" s="1">
+        <f t="shared" si="4"/>
+        <v>5.1663392309968602E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <v>-3</v>
+      </c>
+      <c r="H10" s="1">
+        <f>1.551/2</f>
+        <v>0.77549999999999997</v>
+      </c>
+      <c r="I10" s="1">
+        <f t="shared" si="0"/>
+        <v>7.7549999999999994E-2</v>
+      </c>
+      <c r="J10" s="4">
+        <v>2670</v>
+      </c>
+      <c r="K10" s="1">
+        <f>SUM(J10:J16)/J5</f>
+        <v>8.9800000000000005E-2</v>
+      </c>
+      <c r="L10" s="1">
+        <f t="shared" si="1"/>
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="M10" s="1">
+        <f>SUM(J10:J16)/SUM(J6:J16)</f>
+        <v>7.6830937713894598E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <f t="shared" si="2"/>
+        <v>0.76830937713894598</v>
+      </c>
+      <c r="O10" s="1">
+        <f t="shared" si="3"/>
+        <v>0.54327677062416124</v>
+      </c>
+      <c r="P10" s="1">
+        <f t="shared" si="4"/>
+        <v>-3.0811271348198099</v>
+      </c>
+    </row>
+    <row r="11" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <v>-6</v>
+      </c>
+      <c r="H11">
+        <f>1.098/2</f>
+        <v>0.54900000000000004</v>
+      </c>
+      <c r="I11" s="1">
+        <f t="shared" si="0"/>
+        <v>5.4900000000000004E-2</v>
+      </c>
+      <c r="J11" s="4">
+        <v>1820</v>
+      </c>
+      <c r="K11" s="1">
+        <f>SUM(J11:J16)/J5</f>
+        <v>6.3100000000000003E-2</v>
+      </c>
+      <c r="L11" s="1">
+        <f t="shared" si="1"/>
+        <v>0.63100000000000001</v>
+      </c>
+      <c r="M11" s="1">
+        <f>SUM(J11:J16)/SUM(J6:J16)</f>
+        <v>5.3986995208761122E-2</v>
+      </c>
+      <c r="N11" s="1">
+        <f t="shared" si="2"/>
+        <v>0.53986995208761124</v>
+      </c>
+      <c r="O11" s="1">
+        <f t="shared" si="3"/>
+        <v>0.38174570408000641</v>
+      </c>
+      <c r="P11" s="1">
+        <f t="shared" si="4"/>
+        <v>-6.1460666832832107</v>
+      </c>
+    </row>
+    <row r="12" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>-9</v>
+      </c>
+      <c r="H12" s="1">
+        <f>0.777/2</f>
+        <v>0.38850000000000001</v>
+      </c>
+      <c r="I12" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8850000000000003E-2</v>
+      </c>
+      <c r="J12" s="4">
+        <v>1330</v>
+      </c>
+      <c r="K12" s="1">
+        <f>SUM(J12:J16)/J5</f>
+        <v>4.4900000000000002E-2</v>
+      </c>
+      <c r="L12" s="1">
+        <f t="shared" si="1"/>
+        <v>0.44900000000000001</v>
+      </c>
+      <c r="M12" s="1">
+        <f>SUM(J12:J16)/SUM(J6:J16)</f>
+        <v>3.8415468856947299E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <f t="shared" si="2"/>
+        <v>0.38415468856947299</v>
+      </c>
+      <c r="O12" s="1">
+        <f t="shared" si="3"/>
+        <v>0.27163838531208062</v>
+      </c>
+      <c r="P12" s="1">
+        <f t="shared" si="4"/>
+        <v>-9.1017270480994341</v>
+      </c>
+    </row>
+    <row r="13" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <v>-12</v>
+      </c>
+      <c r="H13">
+        <f>0.55/2</f>
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="I13" s="1">
+        <f t="shared" si="0"/>
+        <v>2.7500000000000004E-2</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1560</v>
+      </c>
+      <c r="K13" s="1">
+        <f>SUM(J13:J16)/J5</f>
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="L13" s="1">
+        <f t="shared" si="1"/>
+        <v>0.31600000000000006</v>
+      </c>
+      <c r="M13" s="1">
+        <f>SUM(J13:J16)/SUM(J6:J16)</f>
+        <v>2.70362765229295E-2</v>
+      </c>
+      <c r="N13" s="1">
+        <f t="shared" si="2"/>
+        <v>0.27036276522929498</v>
+      </c>
+      <c r="O13" s="1">
+        <f t="shared" si="3"/>
+        <v>0.19117534467398098</v>
+      </c>
+      <c r="P13" s="1">
+        <f t="shared" si="4"/>
+        <v>-12.152912215797825</v>
+      </c>
+    </row>
+    <row r="14" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G14">
+        <v>-15</v>
+      </c>
+      <c r="H14">
+        <f>0.39/2</f>
+        <v>0.19500000000000001</v>
+      </c>
+      <c r="I14" s="1">
+        <f t="shared" si="0"/>
+        <v>1.95E-2</v>
+      </c>
+      <c r="J14" s="4">
+        <v>820</v>
+      </c>
+      <c r="K14" s="1">
+        <f>SUM(J14:J16)/J5</f>
+        <v>1.6E-2</v>
+      </c>
+      <c r="L14" s="1">
+        <f t="shared" si="1"/>
+        <v>0.16</v>
+      </c>
+      <c r="M14" s="1">
+        <f>SUM(J14:J16)/SUM(J6:J16)</f>
+        <v>1.3689253935660506E-2</v>
+      </c>
+      <c r="N14" s="1">
+        <f t="shared" si="2"/>
+        <v>0.13689253935660506</v>
+      </c>
+      <c r="O14" s="1">
+        <f t="shared" si="3"/>
+        <v>9.6797642872901768E-2</v>
+      </c>
+      <c r="P14" s="1">
+        <f t="shared" si="4"/>
+        <v>-18.064254215047406</v>
+      </c>
+    </row>
+    <row r="15" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G15">
+        <v>-18</v>
+      </c>
+      <c r="H15">
+        <f>0.276/2</f>
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="I15" s="1">
+        <f>H15/$I$5</f>
+        <v>1.3800000000000002E-2</v>
+      </c>
+      <c r="J15" s="4">
+        <v>390</v>
+      </c>
+      <c r="K15" s="1">
+        <f>SUM(J15:J16)/J6</f>
+        <v>8.580858085808581E-3</v>
+      </c>
+      <c r="L15" s="1">
+        <f t="shared" si="1"/>
+        <v>8.5808580858085806E-2</v>
+      </c>
+      <c r="M15" s="1">
+        <f>SUM(J15:J16)/SUM(J6:J16)</f>
+        <v>6.673511293634497E-3</v>
+      </c>
+      <c r="N15" s="1">
+        <f t="shared" si="2"/>
+        <v>6.6735112936344973E-2</v>
+      </c>
+      <c r="O15" s="1">
+        <f t="shared" si="3"/>
+        <v>4.718885090053962E-2</v>
+      </c>
+      <c r="P15" s="1">
+        <f t="shared" si="4"/>
+        <v>-24.30476181435629</v>
+      </c>
+    </row>
+    <row r="16" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G16">
+        <v>-21</v>
+      </c>
+      <c r="H16" s="1">
+        <f>0.195/2</f>
+        <v>9.7500000000000003E-2</v>
+      </c>
+      <c r="I16" s="1">
+        <f>H16/$I$5</f>
+        <v>9.75E-3</v>
+      </c>
+      <c r="J16" s="4">
+        <v>390</v>
+      </c>
+      <c r="K16" s="1">
+        <f t="shared" ref="K16" si="5">J16/$J$5</f>
+        <v>3.8999999999999998E-3</v>
+      </c>
+      <c r="L16" s="1">
+        <f t="shared" si="1"/>
+        <v>3.9E-2</v>
+      </c>
+      <c r="M16" s="1">
+        <f>SUM(J16)/SUM(J6:J16)</f>
+        <v>3.3367556468172485E-3</v>
+      </c>
+      <c r="N16" s="1">
+        <f t="shared" si="2"/>
+        <v>3.3367556468172486E-2</v>
+      </c>
+      <c r="O16" s="1">
+        <f t="shared" si="3"/>
+        <v>2.359442545026981E-2</v>
+      </c>
+      <c r="P16" s="1">
+        <f t="shared" si="4"/>
+        <v>-30.325361727635915</v>
       </c>
     </row>
     <row r="24" spans="5:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update dBu meter calculation.xlsx
</commit_message>
<xml_diff>
--- a/dBu meter calculation.xlsx
+++ b/dBu meter calculation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodri\Documents\GitHub\DMH-Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4126A16D-EC76-4F97-BEFA-F592ACEC9BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071EA9CC-757C-49F5-B594-6C4801F8AB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{34920A5C-097A-4EEA-8361-CAFEEE971C72}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{34920A5C-097A-4EEA-8361-CAFEEE971C72}"/>
   </bookViews>
   <sheets>
     <sheet name="Out 11v70" sheetId="6" r:id="rId1"/>
@@ -88,7 +88,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.00000E+00"/>
+    <numFmt numFmtId="165" formatCode="0.00000E+00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -115,12 +115,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -135,13 +141,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -151,6 +157,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3175,32 +3182,32 @@
         <f t="shared" ref="I7:I14" si="0">H7/$I$5</f>
         <v>0.21855000000000002</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="9">
         <v>6800</v>
       </c>
       <c r="K7" s="1">
         <f>SUM(J7:J16)/J5</f>
-        <v>0.22925000000000001</v>
+        <v>0.22927</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" ref="L7:L16" si="1">K7*$I$5</f>
-        <v>2.2925</v>
+        <v>2.2927</v>
       </c>
       <c r="M7" s="1">
         <f>SUM(J7:J16)/SUM(J6:J16)</f>
-        <v>0.21848939718846797</v>
+        <v>0.21850429346116823</v>
       </c>
       <c r="N7" s="1">
         <f>M7*$I$5</f>
-        <v>2.1848939718846796</v>
+        <v>2.1850429346116824</v>
       </c>
       <c r="O7" s="1">
         <f>N7/SQRT(2)</f>
-        <v>1.5449533436932668</v>
+        <v>1.5450586762476746</v>
       </c>
       <c r="P7" s="1">
         <f>20*LOG10(O7/0.7746)</f>
-        <v>5.9967575195295293</v>
+        <v>5.9973496900048104</v>
       </c>
     </row>
     <row r="8" spans="7:16" x14ac:dyDescent="0.3">
@@ -3220,27 +3227,27 @@
       </c>
       <c r="K8" s="1">
         <f>SUM(J8:J16)/J5</f>
-        <v>0.16125</v>
+        <v>0.16127</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" si="1"/>
-        <v>1.6125</v>
+        <v>1.6127</v>
       </c>
       <c r="M8" s="1">
         <f>SUM(J8:J16)/SUM(J6:J16)</f>
-        <v>0.15368120085775555</v>
+        <v>0.15369733243111877</v>
       </c>
       <c r="N8" s="1">
         <f t="shared" ref="N8:N16" si="2">M8*$I$5</f>
-        <v>1.5368120085775554</v>
+        <v>1.5369733243111878</v>
       </c>
       <c r="O8" s="1">
         <f t="shared" ref="O8:O16" si="3">N8/SQRT(2)</f>
-        <v>1.0866901926741079</v>
+        <v>1.0868042601232715</v>
       </c>
       <c r="P8" s="1">
         <f t="shared" ref="P8:P16" si="4">20*LOG10(O8/0.7746)</f>
-        <v>2.9405650988344636</v>
+        <v>2.9414767894756464</v>
       </c>
     </row>
     <row r="9" spans="7:16" x14ac:dyDescent="0.3">
@@ -3260,27 +3267,27 @@
       </c>
       <c r="K9" s="1">
         <f>SUM(J9:J16)/J5</f>
-        <v>0.11425</v>
+        <v>0.11427</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="1"/>
-        <v>1.1425000000000001</v>
+        <v>1.1427</v>
       </c>
       <c r="M9" s="1">
         <f>SUM(J9:J16)/SUM(J6:J16)</f>
-        <v>0.10888730045270431</v>
+        <v>0.10890428583681988</v>
       </c>
       <c r="N9" s="1">
         <f t="shared" si="2"/>
-        <v>1.0888730045270432</v>
+        <v>1.0890428583681988</v>
       </c>
       <c r="O9" s="1">
         <f t="shared" si="3"/>
-        <v>0.76994948535204244</v>
+        <v>0.77006959015493415</v>
       </c>
       <c r="P9" s="1">
         <f t="shared" si="4"/>
-        <v>-5.2305192473887568E-2</v>
+        <v>-5.0950381898323259E-2</v>
       </c>
     </row>
     <row r="10" spans="7:16" x14ac:dyDescent="0.3">
@@ -3295,32 +3302,32 @@
         <f t="shared" si="0"/>
         <v>7.7549999999999994E-2</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="9">
         <v>2370</v>
       </c>
       <c r="K10" s="1">
         <f>SUM(J10:J16)/J5</f>
-        <v>8.1250000000000003E-2</v>
+        <v>8.1269999999999995E-2</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="1"/>
-        <v>0.8125</v>
+        <v>0.81269999999999998</v>
       </c>
       <c r="M10" s="1">
         <f>SUM(J10:J16)/SUM(J6:J16)</f>
-        <v>7.7436263998093877E-2</v>
+        <v>7.7453848866354702E-2</v>
       </c>
       <c r="N10" s="1">
         <f t="shared" si="2"/>
-        <v>0.77436263998093879</v>
+        <v>0.77453848866354702</v>
       </c>
       <c r="O10" s="1">
         <f t="shared" si="3"/>
-        <v>0.54755707382803898</v>
+        <v>0.54768141762397393</v>
       </c>
       <c r="P10" s="1">
         <f t="shared" si="4"/>
-        <v>-3.0129619742934031</v>
+        <v>-3.010989734453883</v>
       </c>
     </row>
     <row r="11" spans="7:16" x14ac:dyDescent="0.3">
@@ -3335,32 +3342,32 @@
         <f t="shared" si="0"/>
         <v>5.4900000000000004E-2</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="9">
         <v>1690</v>
       </c>
       <c r="K11" s="1">
         <f>SUM(J11:J16)/J5</f>
-        <v>5.7549999999999997E-2</v>
+        <v>5.7570000000000003E-2</v>
       </c>
       <c r="L11" s="1">
         <f t="shared" si="1"/>
-        <v>0.57550000000000001</v>
+        <v>0.57569999999999999</v>
       </c>
       <c r="M11" s="1">
         <f>SUM(J11:J16)/SUM(J6:J16)</f>
-        <v>5.4848701453419108E-2</v>
+        <v>5.4866716860293346E-2</v>
       </c>
       <c r="N11" s="1">
         <f t="shared" si="2"/>
-        <v>0.54848701453419113</v>
+        <v>0.54866716860293341</v>
       </c>
       <c r="O11" s="1">
         <f t="shared" si="3"/>
-        <v>0.38783888736989097</v>
+        <v>0.387966275533557</v>
       </c>
       <c r="P11" s="1">
         <f t="shared" si="4"/>
-        <v>-6.0085228079954325</v>
+        <v>-6.0056703404078169</v>
       </c>
     </row>
     <row r="12" spans="7:16" x14ac:dyDescent="0.3">
@@ -3375,32 +3382,32 @@
         <f t="shared" si="0"/>
         <v>3.8850000000000003E-2</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="9">
         <v>1200</v>
       </c>
       <c r="K12" s="1">
         <f>SUM(J12:J16)/J5</f>
-        <v>4.0649999999999999E-2</v>
+        <v>4.0669999999999998E-2</v>
       </c>
       <c r="L12" s="1">
         <f t="shared" si="1"/>
-        <v>0.40649999999999997</v>
+        <v>0.40669999999999995</v>
       </c>
       <c r="M12" s="1">
         <f>SUM(J12:J16)/SUM(J6:J16)</f>
-        <v>3.8741958541815585E-2</v>
+        <v>3.8760280957236937E-2</v>
       </c>
       <c r="N12" s="1">
         <f t="shared" si="2"/>
-        <v>0.38741958541815585</v>
+        <v>0.38760280957236937</v>
       </c>
       <c r="O12" s="1">
         <f t="shared" si="3"/>
-        <v>0.27394701601365889</v>
+        <v>0.27407657505558042</v>
       </c>
       <c r="P12" s="1">
         <f t="shared" si="4"/>
-        <v>-9.0282183687099025</v>
+        <v>-9.0241114814187444</v>
       </c>
     </row>
     <row r="13" spans="7:16" x14ac:dyDescent="0.3">
@@ -3415,32 +3422,32 @@
         <f t="shared" si="0"/>
         <v>2.7500000000000004E-2</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="9">
         <v>1430</v>
       </c>
       <c r="K13" s="1">
         <f>SUM(J13:J16)/J5</f>
-        <v>2.8649999999999998E-2</v>
+        <v>2.8670000000000001E-2</v>
       </c>
       <c r="L13" s="1">
         <f t="shared" si="1"/>
-        <v>0.28649999999999998</v>
+        <v>0.28670000000000001</v>
       </c>
       <c r="M13" s="1">
         <f>SUM(J13:J16)/SUM(J6:J16)</f>
-        <v>2.7305218012866332E-2</v>
+        <v>2.7323758422522326E-2</v>
       </c>
       <c r="N13" s="1">
         <f t="shared" si="2"/>
-        <v>0.27305218012866334</v>
+        <v>0.27323758422522326</v>
       </c>
       <c r="O13" s="1">
         <f t="shared" si="3"/>
-        <v>0.19307704818674848</v>
+        <v>0.19320814868068578</v>
       </c>
       <c r="P13" s="1">
         <f t="shared" si="4"/>
-        <v>-12.06693684124347</v>
+        <v>-12.061041070580805</v>
       </c>
     </row>
     <row r="14" spans="7:16" x14ac:dyDescent="0.3">
@@ -3455,32 +3462,32 @@
         <f t="shared" si="0"/>
         <v>1.95E-2</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="9">
         <v>715</v>
       </c>
       <c r="K14" s="1">
         <f>SUM(J14:J16)/J5</f>
-        <v>1.435E-2</v>
+        <v>1.4370000000000001E-2</v>
       </c>
       <c r="L14" s="1">
         <f t="shared" si="1"/>
-        <v>0.14349999999999999</v>
+        <v>0.14369999999999999</v>
       </c>
       <c r="M14" s="1">
         <f>SUM(J14:J16)/SUM(J6:J16)</f>
-        <v>1.3676435549201811E-2</v>
+        <v>1.3695235735320747E-2</v>
       </c>
       <c r="N14" s="1">
         <f t="shared" si="2"/>
-        <v>0.13676435549201812</v>
+        <v>0.13695235735320746</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" si="3"/>
-        <v>9.6707003193013646E-2</v>
+        <v>9.6839940583936329E-2</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" si="4"/>
-        <v>-18.07239134591142</v>
+        <v>-18.060459566825983</v>
       </c>
     </row>
     <row r="15" spans="7:16" x14ac:dyDescent="0.3">
@@ -3496,31 +3503,31 @@
         <v>1.3800000000000002E-2</v>
       </c>
       <c r="J15" s="4">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K15" s="1">
         <f>SUM(J15:J16)/J6</f>
-        <v>8.7804878048780496E-3</v>
+        <v>8.804878048780487E-3</v>
       </c>
       <c r="L15" s="1">
         <f t="shared" si="1"/>
-        <v>8.7804878048780496E-2</v>
+        <v>8.8048780487804873E-2</v>
       </c>
       <c r="M15" s="1">
         <f>SUM(J15:J16)/SUM(J6:J16)</f>
-        <v>6.8620443173695493E-3</v>
+        <v>6.8809743917199575E-3</v>
       </c>
       <c r="N15" s="1">
         <f t="shared" si="2"/>
-        <v>6.8620443173695492E-2</v>
+        <v>6.8809743917199573E-2</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" si="3"/>
-        <v>4.8521980696146216E-2</v>
+        <v>4.8655836535561603E-2</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" si="4"/>
-        <v>-24.062779438686274</v>
+        <v>-24.038850978117715</v>
       </c>
     </row>
     <row r="16" spans="7:16" x14ac:dyDescent="0.3">
@@ -3536,31 +3543,31 @@
         <v>9.75E-3</v>
       </c>
       <c r="J16" s="4">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" ref="K16" si="5">J16/$J$5</f>
-        <v>3.5999999999999999E-3</v>
+        <v>3.6099999999999999E-3</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" si="1"/>
-        <v>3.5999999999999997E-2</v>
+        <v>3.61E-2</v>
       </c>
       <c r="M16" s="1">
         <f>SUM(J16)/SUM(J6:J16)</f>
-        <v>3.4310221586847747E-3</v>
+        <v>3.4404871958599787E-3</v>
       </c>
       <c r="N16" s="1">
         <f t="shared" si="2"/>
-        <v>3.4310221586847746E-2</v>
+        <v>3.4404871958599786E-2</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" si="3"/>
-        <v>2.4260990348073108E-2</v>
+        <v>2.4327918267780801E-2</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" si="4"/>
-        <v>-30.083379351965899</v>
+        <v>-30.05945089139734</v>
       </c>
     </row>
     <row r="19" spans="5:10" x14ac:dyDescent="0.3">
@@ -3569,7 +3576,7 @@
       </c>
       <c r="J19" s="5">
         <f>I5/SUM(J6:J16)</f>
-        <v>9.5306171074577083E-5</v>
+        <v>9.5304354455955087E-5</v>
       </c>
     </row>
     <row r="24" spans="5:10" x14ac:dyDescent="0.3">
@@ -3695,7 +3702,7 @@
         <v>3.2324881425670742</v>
       </c>
       <c r="N8" s="1">
-        <f t="shared" ref="N8:N10" si="2">20*LOG10(M8/0.7746)</f>
+        <f t="shared" ref="N8:N9" si="2">20*LOG10(M8/0.7746)</f>
         <v>12.409188956471892</v>
       </c>
       <c r="O8" t="s">

</xml_diff>